<commit_message>
fix: improve k21 lecture 3 example progression
</commit_message>
<xml_diff>
--- a/src/k21_2026_lecture3/scores.xlsx
+++ b/src/k21_2026_lecture3/scores.xlsx
@@ -14,13 +14,14 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Scores" sheetId="2" r:id="rId4"/>
+    <sheet name="Survey" sheetId="3" r:id="rId6"/>
   </sheets>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>name</t>
   </si>
@@ -41,6 +42,21 @@
   </si>
   <si>
     <t>Eve</t>
+  </si>
+  <si>
+    <t>satisfaction</t>
+  </si>
+  <si>
+    <t>hardest_topic</t>
+  </si>
+  <si>
+    <t>tools</t>
+  </si>
+  <si>
+    <t>MCP</t>
+  </si>
+  <si>
+    <t>guardrails</t>
   </si>
 </sst>
 </file>
@@ -475,4 +491,78 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C6"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>